<commit_message>
TOTAL RH: print as 2 landscape pages
Manual page break before the CARGO CLASSIFICATION section so page 1 is
the weekly blocks/roll-up/remarks/durian tables and page 2 is CARGO +
the full Year x Brand x Size matrix. A4 landscape, 100% scale (fit-to-
page would make Excel ignore the manual break), narrow margins,
print area A:Q. Break row follows CARGO_ROW0 so Rule 1/2 both work.

Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Stock_Daily_Reefer_10-8.xlsx
+++ b/Stock_Daily_Reefer_10-8.xlsx
@@ -13,7 +13,9 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="TOTAL RH" sheetId="4" state="visible" r:id="rId4"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dashboard" sheetId="5" state="visible" r:id="rId5"/>
   </sheets>
-  <definedNames/>
+  <definedNames>
+    <definedName name="_xlnm.Print_Area" localSheetId="3">'TOTAL RH'!$A$1:$Q$59</definedName>
+  </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
 </file>
@@ -7264,7 +7266,12 @@
     <mergeCell ref="B21:B22"/>
     <mergeCell ref="B2:D2"/>
   </mergeCells>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <printOptions horizontalCentered="1"/>
+  <pageMargins left="0.4" right="0.4" top="0.5" bottom="0.5" header="0.5" footer="0.5"/>
+  <pageSetup orientation="landscape" paperSize="9" scale="100"/>
+  <rowBreaks count="1" manualBreakCount="1">
+    <brk id="32" min="0" max="16383" man="1"/>
+  </rowBreaks>
 </worksheet>
 </file>
 

</xml_diff>

<commit_message>
Split TOTAL RH into two sheets: TOTAL RH + YEAR BUILT
User spec: the CARGO CLASSIFICATION section and the full Year x Brand x
Size matrix now live on their own sheet "YEAR BUILT" (starting at A1)
instead of being the lower half of TOTAL RH. Dashboard references into
that section (RF Seasonal 2020-26 card, CARGO cards, current-mix table)
now point at 'YEAR BUILT'. Replaces the previous 2-page print break:
each sheet now prints as one landscape A4 page (fit to page). Verified
cargo/RF Seasonal/mix values unchanged after the move.

Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Stock_Daily_Reefer_10-8.xlsx
+++ b/Stock_Daily_Reefer_10-8.xlsx
@@ -4,17 +4,19 @@
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
-    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="4" autoFilterDateGrouping="1"/>
+    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="5" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Control" sheetId="1" state="visible" r:id="rId1"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="BookingRaw" sheetId="2" state="visible" r:id="rId2"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="StockRaw" sheetId="3" state="visible" r:id="rId3"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="TOTAL RH" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dashboard" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="YEAR BUILT" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dashboard" sheetId="6" state="visible" r:id="rId6"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm.Print_Area" localSheetId="3">'TOTAL RH'!$A$1:$Q$59</definedName>
+    <definedName name="_xlnm.Print_Area" localSheetId="3">'TOTAL RH'!$A$1:$Q$30</definedName>
+    <definedName name="_xlnm.Print_Area" localSheetId="4">'YEAR BUILT'!$A$1:$Q$27</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -290,39 +292,6 @@
       </bottom>
     </border>
     <border>
-      <left style="thin">
-        <color rgb="00BFBFBF"/>
-      </left>
-      <right/>
-      <top/>
-      <bottom/>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="thin">
-        <color rgb="00BFBFBF"/>
-      </left>
-      <right style="thin">
-        <color rgb="00BFBFBF"/>
-      </right>
-      <top/>
-      <bottom/>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="thin">
-        <color rgb="00BFBFBF"/>
-      </left>
-      <right style="thin">
-        <color rgb="00BFBFBF"/>
-      </right>
-      <top/>
-      <bottom style="thin">
-        <color rgb="00BFBFBF"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
       <left/>
       <right/>
       <top style="thin">
@@ -361,6 +330,39 @@
       <top style="thin">
         <color rgb="00BFBFBF"/>
       </top>
+      <bottom style="thin">
+        <color rgb="00BFBFBF"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color rgb="00BFBFBF"/>
+      </left>
+      <right/>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color rgb="00BFBFBF"/>
+      </left>
+      <right style="thin">
+        <color rgb="00BFBFBF"/>
+      </right>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color rgb="00BFBFBF"/>
+      </left>
+      <right style="thin">
+        <color rgb="00BFBFBF"/>
+      </right>
+      <top/>
       <bottom style="thin">
         <color rgb="00BFBFBF"/>
       </bottom>
@@ -543,15 +545,15 @@
       <alignment horizontal="left"/>
     </xf>
     <xf numFmtId="0" fontId="28" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="8" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="9" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="5" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="33" fillId="5" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="9" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="12" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="13" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="30" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -5223,9 +5225,9 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
+    <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:P59"/>
+  <dimension ref="A1:O30"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="4" customWidth="1" min="1" max="1"/>
@@ -5266,7 +5268,6 @@
       <c r="M1" s="1" t="n"/>
       <c r="N1" s="1" t="n"/>
       <c r="O1" s="1" t="n"/>
-      <c r="P1" s="1" t="n"/>
     </row>
     <row r="2" ht="13" customHeight="1">
       <c r="A2" s="1" t="n"/>
@@ -5304,7 +5305,6 @@
           <t>45RE</t>
         </is>
       </c>
-      <c r="P2" s="1" t="n"/>
     </row>
     <row r="3" ht="13" customHeight="1">
       <c r="A3" s="4" t="inlineStr">
@@ -5356,7 +5356,6 @@
         <f>D4</f>
         <v/>
       </c>
-      <c r="P3" s="1" t="n"/>
     </row>
     <row r="4" ht="13" customHeight="1">
       <c r="A4" s="1" t="n"/>
@@ -5400,7 +5399,6 @@
         <f>J4</f>
         <v/>
       </c>
-      <c r="P4" s="1" t="n"/>
     </row>
     <row r="5" ht="13" customHeight="1">
       <c r="A5" s="7">
@@ -5454,7 +5452,6 @@
         <f>SUM(O3:O4)</f>
         <v/>
       </c>
-      <c r="P5" s="1" t="n"/>
     </row>
     <row r="6" ht="13" customHeight="1">
       <c r="A6" s="7">
@@ -5496,7 +5493,6 @@
       <c r="M6" s="1" t="n"/>
       <c r="N6" s="1" t="n"/>
       <c r="O6" s="1" t="n"/>
-      <c r="P6" s="1" t="n"/>
     </row>
     <row r="7" ht="13" customHeight="1">
       <c r="A7" s="7">
@@ -5550,7 +5546,6 @@
           <t>45RE</t>
         </is>
       </c>
-      <c r="P7" s="1" t="n"/>
     </row>
     <row r="8" ht="13" customHeight="1">
       <c r="A8" s="1" t="n"/>
@@ -5596,7 +5591,6 @@
         <f>D5+D6+D7+D9+D11</f>
         <v/>
       </c>
-      <c r="P8" s="1" t="n"/>
     </row>
     <row r="9" ht="13" customHeight="1">
       <c r="A9" s="7">
@@ -5648,7 +5642,6 @@
         <f>J5+J6+J7+J9+J11</f>
         <v/>
       </c>
-      <c r="P9" s="1" t="n"/>
     </row>
     <row r="10" ht="13" customHeight="1">
       <c r="A10" s="1" t="n"/>
@@ -5694,7 +5687,6 @@
         <f>SUM(O8:O9)</f>
         <v/>
       </c>
-      <c r="P10" s="1" t="n"/>
     </row>
     <row r="11" ht="13" customHeight="1">
       <c r="A11" s="7">
@@ -5736,7 +5728,6 @@
       <c r="M11" s="1" t="n"/>
       <c r="N11" s="1" t="n"/>
       <c r="O11" s="1" t="n"/>
-      <c r="P11" s="1" t="n"/>
     </row>
     <row r="12" ht="13" customHeight="1">
       <c r="A12" s="1" t="n"/>
@@ -5784,7 +5775,6 @@
           <t>45RE</t>
         </is>
       </c>
-      <c r="P12" s="1" t="n"/>
     </row>
     <row r="13" ht="13" customHeight="1">
       <c r="A13" s="1" t="n"/>
@@ -5812,7 +5802,6 @@
         <f>D12</f>
         <v/>
       </c>
-      <c r="P13" s="1" t="n"/>
     </row>
     <row r="14" ht="13" customHeight="1">
       <c r="A14" s="14" t="inlineStr">
@@ -5848,7 +5837,6 @@
         <f>J12</f>
         <v/>
       </c>
-      <c r="P14" s="1" t="n"/>
     </row>
     <row r="15" ht="13" customHeight="1">
       <c r="A15" s="1" t="n"/>
@@ -5892,7 +5880,6 @@
         <f>SUM(O13:O14)</f>
         <v/>
       </c>
-      <c r="P15" s="1" t="n"/>
     </row>
     <row r="16" ht="13" customHeight="1">
       <c r="A16" s="1" t="n"/>
@@ -5930,7 +5917,6 @@
       <c r="M16" s="1" t="n"/>
       <c r="N16" s="1" t="n"/>
       <c r="O16" s="1" t="n"/>
-      <c r="P16" s="1" t="n"/>
     </row>
     <row r="17" ht="13" customHeight="1">
       <c r="A17" s="1" t="n"/>
@@ -5968,7 +5954,6 @@
       <c r="M17" s="1" t="n"/>
       <c r="N17" s="1" t="n"/>
       <c r="O17" s="1" t="n"/>
-      <c r="P17" s="1" t="n"/>
     </row>
     <row r="18" ht="13" customHeight="1">
       <c r="A18" s="1" t="n"/>
@@ -5986,7 +5971,6 @@
       <c r="M18" s="1" t="n"/>
       <c r="N18" s="1" t="n"/>
       <c r="O18" s="1" t="n"/>
-      <c r="P18" s="1" t="n"/>
     </row>
     <row r="19" ht="13" customHeight="1">
       <c r="A19" s="1" t="n"/>
@@ -6004,7 +5988,6 @@
       <c r="M19" s="1" t="n"/>
       <c r="N19" s="1" t="n"/>
       <c r="O19" s="1" t="n"/>
-      <c r="P19" s="1" t="n"/>
     </row>
     <row r="20" ht="13" customHeight="1">
       <c r="A20" s="1" t="n"/>
@@ -6030,7 +6013,6 @@
       <c r="M20" s="1" t="n"/>
       <c r="N20" s="1" t="n"/>
       <c r="O20" s="1" t="n"/>
-      <c r="P20" s="1" t="n"/>
     </row>
     <row r="21" ht="13" customHeight="1">
       <c r="A21" s="1" t="n"/>
@@ -6082,7 +6064,6 @@
       <c r="M21" s="1" t="n"/>
       <c r="N21" s="1" t="n"/>
       <c r="O21" s="1" t="n"/>
-      <c r="P21" s="1" t="n"/>
     </row>
     <row r="22" ht="13" customHeight="1">
       <c r="A22" s="1" t="n"/>
@@ -6124,7 +6105,6 @@
       <c r="M22" s="1" t="n"/>
       <c r="N22" s="1" t="n"/>
       <c r="O22" s="1" t="n"/>
-      <c r="P22" s="1" t="n"/>
     </row>
     <row r="23" ht="13" customHeight="1">
       <c r="A23" s="1" t="n"/>
@@ -6158,7 +6138,6 @@
       <c r="M23" s="1" t="n"/>
       <c r="N23" s="1" t="n"/>
       <c r="O23" s="1" t="n"/>
-      <c r="P23" s="1" t="n"/>
     </row>
     <row r="24" ht="13" customHeight="1">
       <c r="A24" s="1" t="n"/>
@@ -6192,7 +6171,6 @@
       <c r="M24" s="1" t="n"/>
       <c r="N24" s="1" t="n"/>
       <c r="O24" s="1" t="n"/>
-      <c r="P24" s="1" t="n"/>
     </row>
     <row r="25" ht="13" customHeight="1">
       <c r="A25" s="1" t="n"/>
@@ -6226,7 +6204,6 @@
       <c r="M25" s="1" t="n"/>
       <c r="N25" s="1" t="n"/>
       <c r="O25" s="1" t="n"/>
-      <c r="P25" s="1" t="n"/>
     </row>
     <row r="26" ht="13" customHeight="1">
       <c r="A26" s="1" t="n"/>
@@ -6260,7 +6237,6 @@
       <c r="M26" s="1" t="n"/>
       <c r="N26" s="1" t="n"/>
       <c r="O26" s="1" t="n"/>
-      <c r="P26" s="1" t="n"/>
     </row>
     <row r="27" ht="13" customHeight="1">
       <c r="A27" s="1" t="n"/>
@@ -6294,7 +6270,6 @@
       <c r="M27" s="1" t="n"/>
       <c r="N27" s="1" t="n"/>
       <c r="O27" s="1" t="n"/>
-      <c r="P27" s="1" t="n"/>
     </row>
     <row r="28" ht="13" customHeight="1">
       <c r="A28" s="1" t="n"/>
@@ -6328,7 +6303,6 @@
       <c r="M28" s="1" t="n"/>
       <c r="N28" s="1" t="n"/>
       <c r="O28" s="1" t="n"/>
-      <c r="P28" s="1" t="n"/>
     </row>
     <row r="29" ht="13" customHeight="1">
       <c r="A29" s="1" t="n"/>
@@ -6366,7 +6340,6 @@
       <c r="M29" s="1" t="n"/>
       <c r="N29" s="1" t="n"/>
       <c r="O29" s="1" t="n"/>
-      <c r="P29" s="1" t="n"/>
     </row>
     <row r="30" ht="13" customHeight="1">
       <c r="A30" s="1" t="n"/>
@@ -6396,886 +6369,883 @@
       <c r="M30" s="1" t="n"/>
       <c r="N30" s="1" t="n"/>
       <c r="O30" s="1" t="n"/>
-      <c r="P30" s="1" t="n"/>
-    </row>
-    <row r="31" ht="13" customHeight="1">
-      <c r="A31" s="1" t="n"/>
-      <c r="B31" s="1" t="n"/>
-      <c r="C31" s="1" t="n"/>
-      <c r="D31" s="1" t="n"/>
-      <c r="E31" s="1" t="n"/>
-      <c r="F31" s="1" t="n"/>
-      <c r="G31" s="1" t="n"/>
-      <c r="H31" s="1" t="n"/>
-      <c r="I31" s="1" t="n"/>
-      <c r="J31" s="1" t="n"/>
-      <c r="K31" s="1" t="n"/>
-      <c r="L31" s="1" t="n"/>
-      <c r="M31" s="1" t="n"/>
-      <c r="N31" s="1" t="n"/>
-      <c r="O31" s="1" t="n"/>
-      <c r="P31" s="1" t="n"/>
-    </row>
-    <row r="32" ht="13" customHeight="1">
-      <c r="A32" s="1" t="n"/>
-      <c r="B32" s="1" t="n"/>
-      <c r="C32" s="1" t="n"/>
-      <c r="D32" s="1" t="n"/>
-      <c r="E32" s="1" t="n"/>
-      <c r="F32" s="1" t="n"/>
-      <c r="G32" s="1" t="n"/>
-      <c r="H32" s="1" t="n"/>
-      <c r="I32" s="1" t="n"/>
-      <c r="J32" s="1" t="n"/>
-      <c r="K32" s="1" t="n"/>
-      <c r="L32" s="1" t="n"/>
-      <c r="M32" s="1" t="n"/>
-      <c r="N32" s="1" t="n"/>
-      <c r="O32" s="1" t="n"/>
-      <c r="P32" s="1" t="n"/>
-    </row>
-    <row r="33" ht="13" customHeight="1">
-      <c r="A33" s="1" t="n"/>
-      <c r="B33" s="21" t="inlineStr">
-        <is>
-          <t>CARGO CLASSIFICATION  (40'RH stock by Built Year, per depot)</t>
-        </is>
-      </c>
-      <c r="C33" s="1" t="n"/>
-      <c r="D33" s="1" t="n"/>
-      <c r="E33" s="1" t="n"/>
-      <c r="F33" s="1" t="n"/>
-      <c r="G33" s="1" t="n"/>
-      <c r="H33" s="1" t="n"/>
-      <c r="I33" s="1" t="n"/>
-      <c r="J33" s="1" t="n"/>
-      <c r="K33" s="1" t="n"/>
-      <c r="L33" s="1" t="n"/>
-      <c r="M33" s="1" t="n"/>
-      <c r="N33" s="1" t="n"/>
-      <c r="O33" s="1" t="n"/>
-      <c r="P33" s="1" t="n"/>
-    </row>
-    <row r="34" ht="13" customHeight="1">
-      <c r="A34" s="1" t="n"/>
-      <c r="B34" s="22" t="inlineStr">
-        <is>
-          <t>BKK27 DURIAN  (2021-2026)</t>
-        </is>
-      </c>
-      <c r="C34" s="23" t="n"/>
-      <c r="D34" s="23" t="n"/>
-      <c r="E34" s="1" t="n"/>
-      <c r="F34" s="22" t="inlineStr">
-        <is>
-          <t>BKK27 NON DURIAN  (≤ 2020)</t>
-        </is>
-      </c>
-      <c r="G34" s="23" t="n"/>
-      <c r="H34" s="23" t="n"/>
-      <c r="I34" s="1" t="n"/>
-      <c r="J34" s="22" t="inlineStr">
-        <is>
-          <t>LCH27 DURIAN  (2021-2026)</t>
-        </is>
-      </c>
-      <c r="K34" s="23" t="n"/>
-      <c r="L34" s="23" t="n"/>
-      <c r="M34" s="1" t="n"/>
-      <c r="N34" s="22" t="inlineStr">
-        <is>
-          <t>LCH27 NON DURIAN  (≤ 2020)</t>
-        </is>
-      </c>
-      <c r="O34" s="23" t="n"/>
-      <c r="P34" s="23" t="n"/>
-    </row>
-    <row r="35" ht="13" customHeight="1">
-      <c r="A35" s="1" t="n"/>
-      <c r="B35" s="24">
-        <f>SUM(D42:D47)+SUM(F42:F47)+SUM(H42:H47)</f>
-        <v/>
-      </c>
-      <c r="C35" s="23" t="n"/>
-      <c r="D35" s="23" t="n"/>
-      <c r="E35" s="1" t="n"/>
-      <c r="F35" s="24">
-        <f>SUM(D48:D58)+SUM(F48:F58)+SUM(H48:H58)</f>
-        <v/>
-      </c>
-      <c r="G35" s="23" t="n"/>
-      <c r="H35" s="23" t="n"/>
-      <c r="I35" s="1" t="n"/>
-      <c r="J35" s="25">
-        <f>SUM(L42:L47)+SUM(N42:N47)+SUM(P42:P47)</f>
-        <v/>
-      </c>
-      <c r="K35" s="23" t="n"/>
-      <c r="L35" s="23" t="n"/>
-      <c r="M35" s="1" t="n"/>
-      <c r="N35" s="25">
-        <f>SUM(L48:L58)+SUM(N48:N58)+SUM(P48:P58)</f>
-        <v/>
-      </c>
-      <c r="O35" s="23" t="n"/>
-      <c r="P35" s="23" t="n"/>
-    </row>
-    <row r="36" ht="13" customHeight="1">
-      <c r="A36" s="1" t="n"/>
-      <c r="B36" s="26" t="inlineStr">
-        <is>
-          <t>40'RH stock</t>
-        </is>
-      </c>
-      <c r="C36" s="23" t="n"/>
-      <c r="D36" s="23" t="n"/>
-      <c r="E36" s="1" t="n"/>
-      <c r="F36" s="26" t="inlineStr">
-        <is>
-          <t>40'RH stock</t>
-        </is>
-      </c>
-      <c r="G36" s="23" t="n"/>
-      <c r="H36" s="23" t="n"/>
-      <c r="I36" s="1" t="n"/>
-      <c r="J36" s="26" t="inlineStr">
-        <is>
-          <t>40'RH stock</t>
-        </is>
-      </c>
-      <c r="K36" s="23" t="n"/>
-      <c r="L36" s="23" t="n"/>
-      <c r="M36" s="1" t="n"/>
-      <c r="N36" s="26" t="inlineStr">
-        <is>
-          <t>40'RH stock</t>
-        </is>
-      </c>
-      <c r="O36" s="23" t="n"/>
-      <c r="P36" s="23" t="n"/>
-    </row>
-    <row r="37" ht="13" customHeight="1">
-      <c r="A37" s="1" t="n"/>
-      <c r="B37" s="1" t="n"/>
-      <c r="C37" s="1" t="n"/>
-      <c r="D37" s="1" t="n"/>
-      <c r="E37" s="1" t="n"/>
-      <c r="F37" s="1" t="n"/>
-      <c r="G37" s="1" t="n"/>
-      <c r="H37" s="1" t="n"/>
-      <c r="I37" s="1" t="n"/>
-      <c r="J37" s="1" t="n"/>
-      <c r="K37" s="1" t="n"/>
-      <c r="L37" s="1" t="n"/>
-      <c r="M37" s="1" t="n"/>
-      <c r="N37" s="1" t="n"/>
-      <c r="O37" s="1" t="n"/>
-      <c r="P37" s="1" t="n"/>
-    </row>
-    <row r="38" ht="13" customHeight="1">
-      <c r="A38" s="1" t="n"/>
-      <c r="B38" s="1" t="n"/>
-      <c r="C38" s="1" t="n"/>
-      <c r="D38" s="1" t="n"/>
-      <c r="E38" s="1" t="n"/>
-      <c r="F38" s="1" t="n"/>
-      <c r="G38" s="1" t="n"/>
-      <c r="H38" s="1" t="n"/>
-      <c r="I38" s="1" t="n"/>
-      <c r="J38" s="1" t="n"/>
-      <c r="K38" s="1" t="n"/>
-      <c r="L38" s="1" t="n"/>
-      <c r="M38" s="1" t="n"/>
-      <c r="N38" s="1" t="n"/>
-      <c r="O38" s="1" t="n"/>
-      <c r="P38" s="1" t="n"/>
-    </row>
-    <row r="39" ht="13" customHeight="1">
-      <c r="A39" s="1" t="n"/>
-      <c r="B39" s="3" t="inlineStr">
-        <is>
-          <t>BKK27 / BC2  —  Stock by Built Year x Brand x Size</t>
-        </is>
-      </c>
-      <c r="C39" s="56" t="n"/>
-      <c r="D39" s="56" t="n"/>
-      <c r="E39" s="56" t="n"/>
-      <c r="F39" s="56" t="n"/>
-      <c r="G39" s="56" t="n"/>
-      <c r="H39" s="57" t="n"/>
-      <c r="I39" s="1" t="n"/>
-      <c r="J39" s="3" t="inlineStr">
-        <is>
-          <t>LCH27 / HAST  —  Stock by Built Year x Brand x Size</t>
-        </is>
-      </c>
-      <c r="K39" s="56" t="n"/>
-      <c r="L39" s="56" t="n"/>
-      <c r="M39" s="56" t="n"/>
-      <c r="N39" s="56" t="n"/>
-      <c r="O39" s="56" t="n"/>
-      <c r="P39" s="57" t="n"/>
-    </row>
-    <row r="40" ht="26" customHeight="1">
-      <c r="A40" s="1" t="n"/>
-      <c r="B40" s="18" t="inlineStr">
-        <is>
-          <t>YEAR
-BUILT</t>
-        </is>
-      </c>
-      <c r="C40" s="4" t="inlineStr">
-        <is>
-          <t>CARRIER</t>
-        </is>
-      </c>
-      <c r="D40" s="57" t="n"/>
-      <c r="E40" s="4" t="inlineStr">
-        <is>
-          <t>DAIKIN</t>
-        </is>
-      </c>
-      <c r="F40" s="57" t="n"/>
-      <c r="G40" s="4" t="inlineStr">
-        <is>
-          <t>THERMO KING</t>
-        </is>
-      </c>
-      <c r="H40" s="57" t="n"/>
-      <c r="I40" s="1" t="n"/>
-      <c r="J40" s="18" t="inlineStr">
-        <is>
-          <t>YEAR
-BUILT</t>
-        </is>
-      </c>
-      <c r="K40" s="4" t="inlineStr">
-        <is>
-          <t>CARRIER</t>
-        </is>
-      </c>
-      <c r="L40" s="57" t="n"/>
-      <c r="M40" s="4" t="inlineStr">
-        <is>
-          <t>DAIKIN</t>
-        </is>
-      </c>
-      <c r="N40" s="57" t="n"/>
-      <c r="O40" s="4" t="inlineStr">
-        <is>
-          <t>THERMO KING</t>
-        </is>
-      </c>
-      <c r="P40" s="57" t="n"/>
-    </row>
-    <row r="41" ht="13" customHeight="1">
-      <c r="A41" s="1" t="n"/>
-      <c r="B41" s="60" t="n"/>
-      <c r="C41" s="28" t="inlineStr">
-        <is>
-          <t>20'RE</t>
-        </is>
-      </c>
-      <c r="D41" s="28" t="inlineStr">
-        <is>
-          <t>40'RH</t>
-        </is>
-      </c>
-      <c r="E41" s="28" t="inlineStr">
-        <is>
-          <t>20'RE</t>
-        </is>
-      </c>
-      <c r="F41" s="28" t="inlineStr">
-        <is>
-          <t>40'RH</t>
-        </is>
-      </c>
-      <c r="G41" s="28" t="inlineStr">
-        <is>
-          <t>20'RE</t>
-        </is>
-      </c>
-      <c r="H41" s="28" t="inlineStr">
-        <is>
-          <t>40'RH</t>
-        </is>
-      </c>
-      <c r="I41" s="1" t="n"/>
-      <c r="J41" s="60" t="n"/>
-      <c r="K41" s="28" t="inlineStr">
-        <is>
-          <t>20'RE</t>
-        </is>
-      </c>
-      <c r="L41" s="28" t="inlineStr">
-        <is>
-          <t>40'RH</t>
-        </is>
-      </c>
-      <c r="M41" s="28" t="inlineStr">
-        <is>
-          <t>20'RE</t>
-        </is>
-      </c>
-      <c r="N41" s="28" t="inlineStr">
-        <is>
-          <t>40'RH</t>
-        </is>
-      </c>
-      <c r="O41" s="28" t="inlineStr">
-        <is>
-          <t>20'RE</t>
-        </is>
-      </c>
-      <c r="P41" s="28" t="inlineStr">
-        <is>
-          <t>40'RH</t>
-        </is>
-      </c>
-    </row>
-    <row r="42" ht="13" customHeight="1">
-      <c r="A42" s="1" t="n"/>
-      <c r="B42" s="29" t="n">
-        <v>2026</v>
-      </c>
-      <c r="C42" s="30" t="n"/>
-      <c r="D42" s="30" t="n"/>
-      <c r="E42" s="30" t="n"/>
-      <c r="F42" s="30" t="n"/>
-      <c r="G42" s="30" t="n"/>
-      <c r="H42" s="30" t="n"/>
-      <c r="I42" s="1" t="n"/>
-      <c r="J42" s="29" t="n">
-        <v>2026</v>
-      </c>
-      <c r="K42" s="30" t="n"/>
-      <c r="L42" s="30" t="n"/>
-      <c r="M42" s="30" t="n"/>
-      <c r="N42" s="30" t="n"/>
-      <c r="O42" s="30" t="n"/>
-      <c r="P42" s="30" t="n"/>
-    </row>
-    <row r="43" ht="13" customHeight="1">
-      <c r="A43" s="1" t="n"/>
-      <c r="B43" s="29" t="n">
-        <v>2025</v>
-      </c>
-      <c r="C43" s="30" t="n"/>
-      <c r="D43" s="30" t="n">
-        <v>3</v>
-      </c>
-      <c r="E43" s="30" t="n">
-        <v>2</v>
-      </c>
-      <c r="F43" s="30" t="n"/>
-      <c r="G43" s="30" t="n"/>
-      <c r="H43" s="30" t="n">
-        <v>1</v>
-      </c>
-      <c r="I43" s="1" t="n"/>
-      <c r="J43" s="29" t="n">
-        <v>2025</v>
-      </c>
-      <c r="K43" s="30" t="n"/>
-      <c r="L43" s="30" t="n">
-        <v>8</v>
-      </c>
-      <c r="M43" s="30" t="n"/>
-      <c r="N43" s="30" t="n"/>
-      <c r="O43" s="30" t="n"/>
-      <c r="P43" s="30" t="n"/>
-    </row>
-    <row r="44" ht="13" customHeight="1">
-      <c r="A44" s="1" t="n"/>
-      <c r="B44" s="29" t="n">
-        <v>2024</v>
-      </c>
-      <c r="C44" s="30" t="n"/>
-      <c r="D44" s="30" t="n"/>
-      <c r="E44" s="30" t="n"/>
-      <c r="F44" s="30" t="n"/>
-      <c r="G44" s="30" t="n"/>
-      <c r="H44" s="30" t="n"/>
-      <c r="I44" s="1" t="n"/>
-      <c r="J44" s="29" t="n">
-        <v>2024</v>
-      </c>
-      <c r="K44" s="30" t="n"/>
-      <c r="L44" s="30" t="n"/>
-      <c r="M44" s="30" t="n"/>
-      <c r="N44" s="30" t="n"/>
-      <c r="O44" s="30" t="n"/>
-      <c r="P44" s="30" t="n"/>
-    </row>
-    <row r="45" ht="13" customHeight="1">
-      <c r="A45" s="1" t="n"/>
-      <c r="B45" s="29" t="n">
-        <v>2023</v>
-      </c>
-      <c r="C45" s="30" t="n"/>
-      <c r="D45" s="30" t="n">
-        <v>1</v>
-      </c>
-      <c r="E45" s="30" t="n"/>
-      <c r="F45" s="30" t="n"/>
-      <c r="G45" s="30" t="n"/>
-      <c r="H45" s="30" t="n"/>
-      <c r="I45" s="1" t="n"/>
-      <c r="J45" s="29" t="n">
-        <v>2023</v>
-      </c>
-      <c r="K45" s="30" t="n"/>
-      <c r="L45" s="30" t="n">
-        <v>2</v>
-      </c>
-      <c r="M45" s="30" t="n"/>
-      <c r="N45" s="30" t="n"/>
-      <c r="O45" s="30" t="n"/>
-      <c r="P45" s="30" t="n"/>
-    </row>
-    <row r="46" ht="13" customHeight="1">
-      <c r="A46" s="1" t="n"/>
-      <c r="B46" s="29" t="n">
-        <v>2022</v>
-      </c>
-      <c r="C46" s="30" t="n"/>
-      <c r="D46" s="30" t="n"/>
-      <c r="E46" s="30" t="n"/>
-      <c r="F46" s="30" t="n"/>
-      <c r="G46" s="30" t="n"/>
-      <c r="H46" s="30" t="n"/>
-      <c r="I46" s="1" t="n"/>
-      <c r="J46" s="29" t="n">
-        <v>2022</v>
-      </c>
-      <c r="K46" s="30" t="n"/>
-      <c r="L46" s="30" t="n"/>
-      <c r="M46" s="30" t="n"/>
-      <c r="N46" s="30" t="n"/>
-      <c r="O46" s="30" t="n"/>
-      <c r="P46" s="30" t="n"/>
-    </row>
-    <row r="47" ht="13" customHeight="1">
-      <c r="A47" s="1" t="n"/>
-      <c r="B47" s="29" t="n">
-        <v>2021</v>
-      </c>
-      <c r="C47" s="30" t="n">
-        <v>8</v>
-      </c>
-      <c r="D47" s="30" t="n">
-        <v>6</v>
-      </c>
-      <c r="E47" s="30" t="n"/>
-      <c r="F47" s="30" t="n"/>
-      <c r="G47" s="30" t="n"/>
-      <c r="H47" s="30" t="n"/>
-      <c r="I47" s="1" t="n"/>
-      <c r="J47" s="29" t="n">
-        <v>2021</v>
-      </c>
-      <c r="K47" s="30" t="n">
-        <v>2</v>
-      </c>
-      <c r="L47" s="30" t="n">
-        <v>3</v>
-      </c>
-      <c r="M47" s="30" t="n"/>
-      <c r="N47" s="30" t="n"/>
-      <c r="O47" s="30" t="n"/>
-      <c r="P47" s="30" t="n"/>
-    </row>
-    <row r="48" ht="13" customHeight="1">
-      <c r="A48" s="1" t="n"/>
-      <c r="B48" s="31" t="n">
-        <v>2020</v>
-      </c>
-      <c r="C48" s="32" t="n">
-        <v>1</v>
-      </c>
-      <c r="D48" s="32" t="n">
-        <v>5</v>
-      </c>
-      <c r="E48" s="32" t="n"/>
-      <c r="F48" s="32" t="n"/>
-      <c r="G48" s="32" t="n"/>
-      <c r="H48" s="32" t="n"/>
-      <c r="I48" s="1" t="n"/>
-      <c r="J48" s="31" t="n">
-        <v>2020</v>
-      </c>
-      <c r="K48" s="32" t="n"/>
-      <c r="L48" s="32" t="n">
-        <v>11</v>
-      </c>
-      <c r="M48" s="32" t="n"/>
-      <c r="N48" s="32" t="n"/>
-      <c r="O48" s="32" t="n"/>
-      <c r="P48" s="32" t="n">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="49" ht="13" customHeight="1">
-      <c r="A49" s="1" t="n"/>
-      <c r="B49" s="31" t="n">
-        <v>2019</v>
-      </c>
-      <c r="C49" s="32" t="n">
-        <v>3</v>
-      </c>
-      <c r="D49" s="32" t="n">
-        <v>5</v>
-      </c>
-      <c r="E49" s="32" t="n"/>
-      <c r="F49" s="32" t="n"/>
-      <c r="G49" s="32" t="n"/>
-      <c r="H49" s="32" t="n"/>
-      <c r="I49" s="1" t="n"/>
-      <c r="J49" s="31" t="n">
-        <v>2019</v>
-      </c>
-      <c r="K49" s="32" t="n"/>
-      <c r="L49" s="32" t="n">
-        <v>8</v>
-      </c>
-      <c r="M49" s="32" t="n"/>
-      <c r="N49" s="32" t="n"/>
-      <c r="O49" s="32" t="n"/>
-      <c r="P49" s="32" t="n"/>
-    </row>
-    <row r="50" ht="13" customHeight="1">
-      <c r="A50" s="1" t="n"/>
-      <c r="B50" s="31" t="n">
-        <v>2018</v>
-      </c>
-      <c r="C50" s="32" t="n">
-        <v>1</v>
-      </c>
-      <c r="D50" s="32" t="n"/>
-      <c r="E50" s="32" t="n"/>
-      <c r="F50" s="32" t="n"/>
-      <c r="G50" s="32" t="n"/>
-      <c r="H50" s="32" t="n"/>
-      <c r="I50" s="1" t="n"/>
-      <c r="J50" s="31" t="n">
-        <v>2018</v>
-      </c>
-      <c r="K50" s="32" t="n"/>
-      <c r="L50" s="32" t="n"/>
-      <c r="M50" s="32" t="n"/>
-      <c r="N50" s="32" t="n"/>
-      <c r="O50" s="32" t="n"/>
-      <c r="P50" s="32" t="n"/>
-    </row>
-    <row r="51" ht="13" customHeight="1">
-      <c r="A51" s="1" t="n"/>
-      <c r="B51" s="31" t="n">
-        <v>2017</v>
-      </c>
-      <c r="C51" s="32" t="n">
-        <v>2</v>
-      </c>
-      <c r="D51" s="32" t="n">
-        <v>1</v>
-      </c>
-      <c r="E51" s="32" t="n"/>
-      <c r="F51" s="32" t="n"/>
-      <c r="G51" s="32" t="n"/>
-      <c r="H51" s="32" t="n"/>
-      <c r="I51" s="1" t="n"/>
-      <c r="J51" s="31" t="n">
-        <v>2017</v>
-      </c>
-      <c r="K51" s="32" t="n">
-        <v>2</v>
-      </c>
-      <c r="L51" s="32" t="n">
-        <v>2</v>
-      </c>
-      <c r="M51" s="32" t="n"/>
-      <c r="N51" s="32" t="n"/>
-      <c r="O51" s="32" t="n"/>
-      <c r="P51" s="32" t="n"/>
-    </row>
-    <row r="52" ht="13" customHeight="1">
-      <c r="A52" s="1" t="n"/>
-      <c r="B52" s="31" t="n">
-        <v>2016</v>
-      </c>
-      <c r="C52" s="32" t="n">
-        <v>2</v>
-      </c>
-      <c r="D52" s="32" t="n">
-        <v>3</v>
-      </c>
-      <c r="E52" s="32" t="n">
-        <v>2</v>
-      </c>
-      <c r="F52" s="32" t="n"/>
-      <c r="G52" s="32" t="n"/>
-      <c r="H52" s="32" t="n"/>
-      <c r="I52" s="1" t="n"/>
-      <c r="J52" s="31" t="n">
-        <v>2016</v>
-      </c>
-      <c r="K52" s="32" t="n"/>
-      <c r="L52" s="32" t="n"/>
-      <c r="M52" s="32" t="n"/>
-      <c r="N52" s="32" t="n"/>
-      <c r="O52" s="32" t="n"/>
-      <c r="P52" s="32" t="n"/>
-    </row>
-    <row r="53" ht="13" customHeight="1">
-      <c r="A53" s="1" t="n"/>
-      <c r="B53" s="33" t="n">
-        <v>2015</v>
-      </c>
-      <c r="C53" s="34" t="n"/>
-      <c r="D53" s="34" t="n">
-        <v>3</v>
-      </c>
-      <c r="E53" s="34" t="n">
-        <v>2</v>
-      </c>
-      <c r="F53" s="34" t="n"/>
-      <c r="G53" s="34" t="n"/>
-      <c r="H53" s="34" t="n"/>
-      <c r="I53" s="1" t="n"/>
-      <c r="J53" s="33" t="n">
-        <v>2015</v>
-      </c>
-      <c r="K53" s="34" t="n"/>
-      <c r="L53" s="34" t="n">
-        <v>2</v>
-      </c>
-      <c r="M53" s="34" t="n"/>
-      <c r="N53" s="34" t="n"/>
-      <c r="O53" s="34" t="n"/>
-      <c r="P53" s="34" t="n"/>
-    </row>
-    <row r="54" ht="13" customHeight="1">
-      <c r="A54" s="1" t="n"/>
-      <c r="B54" s="33" t="n">
-        <v>2014</v>
-      </c>
-      <c r="C54" s="34" t="n">
-        <v>2</v>
-      </c>
-      <c r="D54" s="34" t="n"/>
-      <c r="E54" s="34" t="n"/>
-      <c r="F54" s="34" t="n"/>
-      <c r="G54" s="34" t="n"/>
-      <c r="H54" s="34" t="n"/>
-      <c r="I54" s="1" t="n"/>
-      <c r="J54" s="33" t="n">
-        <v>2014</v>
-      </c>
-      <c r="K54" s="34" t="n"/>
-      <c r="L54" s="34" t="n">
-        <v>5</v>
-      </c>
-      <c r="M54" s="34" t="n"/>
-      <c r="N54" s="34" t="n"/>
-      <c r="O54" s="34" t="n"/>
-      <c r="P54" s="34" t="n"/>
-    </row>
-    <row r="55" ht="13" customHeight="1">
-      <c r="A55" s="1" t="n"/>
-      <c r="B55" s="33" t="n">
-        <v>2013</v>
-      </c>
-      <c r="C55" s="34" t="n">
-        <v>1</v>
-      </c>
-      <c r="D55" s="34" t="n"/>
-      <c r="E55" s="34" t="n">
-        <v>4</v>
-      </c>
-      <c r="F55" s="34" t="n">
-        <v>3</v>
-      </c>
-      <c r="G55" s="34" t="n">
-        <v>2</v>
-      </c>
-      <c r="H55" s="34" t="n">
-        <v>1</v>
-      </c>
-      <c r="I55" s="1" t="n"/>
-      <c r="J55" s="33" t="n">
-        <v>2013</v>
-      </c>
-      <c r="K55" s="34" t="n"/>
-      <c r="L55" s="34" t="n"/>
-      <c r="M55" s="34" t="n">
-        <v>2</v>
-      </c>
-      <c r="N55" s="34" t="n">
-        <v>2</v>
-      </c>
-      <c r="O55" s="34" t="n"/>
-      <c r="P55" s="34" t="n"/>
-    </row>
-    <row r="56" ht="13" customHeight="1">
-      <c r="A56" s="1" t="n"/>
-      <c r="B56" s="33" t="n">
-        <v>2012</v>
-      </c>
-      <c r="C56" s="34" t="n">
-        <v>1</v>
-      </c>
-      <c r="D56" s="34" t="n">
-        <v>2</v>
-      </c>
-      <c r="E56" s="34" t="n"/>
-      <c r="F56" s="34" t="n"/>
-      <c r="G56" s="34" t="n"/>
-      <c r="H56" s="34" t="n"/>
-      <c r="I56" s="1" t="n"/>
-      <c r="J56" s="33" t="n">
-        <v>2012</v>
-      </c>
-      <c r="K56" s="34" t="n"/>
-      <c r="L56" s="34" t="n">
-        <v>3</v>
-      </c>
-      <c r="M56" s="34" t="n">
-        <v>1</v>
-      </c>
-      <c r="N56" s="34" t="n"/>
-      <c r="O56" s="34" t="n"/>
-      <c r="P56" s="34" t="n"/>
-    </row>
-    <row r="57" ht="13" customHeight="1">
-      <c r="A57" s="1" t="n"/>
-      <c r="B57" s="33" t="n">
-        <v>2011</v>
-      </c>
-      <c r="C57" s="34" t="n"/>
-      <c r="D57" s="34" t="n"/>
-      <c r="E57" s="34" t="n"/>
-      <c r="F57" s="34" t="n">
-        <v>3</v>
-      </c>
-      <c r="G57" s="34" t="n"/>
-      <c r="H57" s="34" t="n"/>
-      <c r="I57" s="1" t="n"/>
-      <c r="J57" s="33" t="n">
-        <v>2011</v>
-      </c>
-      <c r="K57" s="34" t="n"/>
-      <c r="L57" s="34" t="n"/>
-      <c r="M57" s="34" t="n"/>
-      <c r="N57" s="34" t="n">
-        <v>5</v>
-      </c>
-      <c r="O57" s="34" t="n"/>
-      <c r="P57" s="34" t="n"/>
-    </row>
-    <row r="58" ht="13" customHeight="1">
-      <c r="A58" s="1" t="n"/>
-      <c r="B58" s="35" t="n">
-        <v>2010</v>
-      </c>
-      <c r="C58" s="36" t="n"/>
-      <c r="D58" s="36" t="n">
-        <v>1</v>
-      </c>
-      <c r="E58" s="36" t="n"/>
-      <c r="F58" s="36" t="n"/>
-      <c r="G58" s="36" t="n"/>
-      <c r="H58" s="36" t="n"/>
-      <c r="I58" s="1" t="n"/>
-      <c r="J58" s="35" t="n">
-        <v>2010</v>
-      </c>
-      <c r="K58" s="36" t="n"/>
-      <c r="L58" s="36" t="n">
-        <v>1</v>
-      </c>
-      <c r="M58" s="36" t="n"/>
-      <c r="N58" s="36" t="n"/>
-      <c r="O58" s="36" t="n"/>
-      <c r="P58" s="36" t="n"/>
-    </row>
-    <row r="59" ht="13" customHeight="1">
-      <c r="A59" s="1" t="n"/>
-      <c r="B59" s="13" t="inlineStr">
-        <is>
-          <t>GTTL</t>
-        </is>
-      </c>
-      <c r="C59" s="13" t="n">
-        <v>21</v>
-      </c>
-      <c r="D59" s="13" t="n">
-        <v>30</v>
-      </c>
-      <c r="E59" s="13" t="n">
-        <v>10</v>
-      </c>
-      <c r="F59" s="13" t="n">
-        <v>6</v>
-      </c>
-      <c r="G59" s="13" t="n">
-        <v>2</v>
-      </c>
-      <c r="H59" s="13" t="n">
-        <v>2</v>
-      </c>
-      <c r="I59" s="1" t="n"/>
-      <c r="J59" s="13" t="inlineStr">
-        <is>
-          <t>GTTL</t>
-        </is>
-      </c>
-      <c r="K59" s="13" t="n">
-        <v>4</v>
-      </c>
-      <c r="L59" s="13" t="n">
-        <v>45</v>
-      </c>
-      <c r="M59" s="13" t="n">
-        <v>3</v>
-      </c>
-      <c r="N59" s="13" t="n">
-        <v>7</v>
-      </c>
-      <c r="O59" s="13" t="n"/>
-      <c r="P59" s="13" t="n">
-        <v>1</v>
-      </c>
     </row>
   </sheetData>
-  <mergeCells count="17">
-    <mergeCell ref="J40:J41"/>
-    <mergeCell ref="J39:P39"/>
-    <mergeCell ref="M40:N40"/>
-    <mergeCell ref="B39:H39"/>
-    <mergeCell ref="O40:P40"/>
+  <mergeCells count="7">
+    <mergeCell ref="A1:K1"/>
     <mergeCell ref="H20:K20"/>
-    <mergeCell ref="A1:K1"/>
-    <mergeCell ref="E40:F40"/>
     <mergeCell ref="H2:J2"/>
     <mergeCell ref="H21:H22"/>
-    <mergeCell ref="C40:D40"/>
     <mergeCell ref="B20:E20"/>
-    <mergeCell ref="G40:H40"/>
-    <mergeCell ref="B40:B41"/>
-    <mergeCell ref="K40:L40"/>
     <mergeCell ref="B21:B22"/>
     <mergeCell ref="B2:D2"/>
   </mergeCells>
   <printOptions horizontalCentered="1"/>
   <pageMargins left="0.4" right="0.4" top="0.5" bottom="0.5" header="0.5" footer="0.5"/>
-  <pageSetup orientation="landscape" paperSize="9" scale="100"/>
-  <rowBreaks count="1" manualBreakCount="1">
-    <brk id="32" min="0" max="16383" man="1"/>
-  </rowBreaks>
+  <pageSetup orientation="landscape" paperSize="9" fitToHeight="1" fitToWidth="1"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr fitToPage="1"/>
+  </sheetPr>
+  <dimension ref="A1:P27"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="4" customWidth="1" min="1" max="1"/>
+    <col width="8" customWidth="1" min="2" max="2"/>
+    <col width="8" customWidth="1" min="3" max="3"/>
+    <col width="8" customWidth="1" min="4" max="4"/>
+    <col width="8" customWidth="1" min="5" max="5"/>
+    <col width="8" customWidth="1" min="6" max="6"/>
+    <col width="8" customWidth="1" min="7" max="7"/>
+    <col width="8" customWidth="1" min="8" max="8"/>
+    <col width="8" customWidth="1" min="9" max="9"/>
+    <col width="8" customWidth="1" min="10" max="10"/>
+    <col width="8" customWidth="1" min="11" max="11"/>
+    <col width="8" customWidth="1" min="12" max="12"/>
+    <col width="8" customWidth="1" min="13" max="13"/>
+    <col width="8" customWidth="1" min="14" max="14"/>
+    <col width="8" customWidth="1" min="15" max="15"/>
+    <col width="8" customWidth="1" min="16" max="16"/>
+    <col width="8" customWidth="1" min="17" max="17"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="13" customHeight="1">
+      <c r="A1" s="1" t="n"/>
+      <c r="B1" s="21" t="inlineStr">
+        <is>
+          <t>CARGO CLASSIFICATION  (40'RH stock by Built Year, per depot)</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="n"/>
+      <c r="D1" s="1" t="n"/>
+      <c r="E1" s="1" t="n"/>
+      <c r="F1" s="1" t="n"/>
+      <c r="G1" s="1" t="n"/>
+      <c r="H1" s="1" t="n"/>
+      <c r="I1" s="1" t="n"/>
+      <c r="J1" s="1" t="n"/>
+      <c r="K1" s="1" t="n"/>
+      <c r="L1" s="1" t="n"/>
+      <c r="M1" s="1" t="n"/>
+      <c r="N1" s="1" t="n"/>
+      <c r="O1" s="1" t="n"/>
+      <c r="P1" s="1" t="n"/>
+    </row>
+    <row r="2" ht="13" customHeight="1">
+      <c r="A2" s="1" t="n"/>
+      <c r="B2" s="22" t="inlineStr">
+        <is>
+          <t>BKK27 DURIAN  (2021-2026)</t>
+        </is>
+      </c>
+      <c r="C2" s="23" t="n"/>
+      <c r="D2" s="23" t="n"/>
+      <c r="E2" s="1" t="n"/>
+      <c r="F2" s="22" t="inlineStr">
+        <is>
+          <t>BKK27 NON DURIAN  (≤ 2020)</t>
+        </is>
+      </c>
+      <c r="G2" s="23" t="n"/>
+      <c r="H2" s="23" t="n"/>
+      <c r="I2" s="1" t="n"/>
+      <c r="J2" s="22" t="inlineStr">
+        <is>
+          <t>LCH27 DURIAN  (2021-2026)</t>
+        </is>
+      </c>
+      <c r="K2" s="23" t="n"/>
+      <c r="L2" s="23" t="n"/>
+      <c r="M2" s="1" t="n"/>
+      <c r="N2" s="22" t="inlineStr">
+        <is>
+          <t>LCH27 NON DURIAN  (≤ 2020)</t>
+        </is>
+      </c>
+      <c r="O2" s="23" t="n"/>
+      <c r="P2" s="23" t="n"/>
+    </row>
+    <row r="3" ht="13" customHeight="1">
+      <c r="A3" s="1" t="n"/>
+      <c r="B3" s="24">
+        <f>SUM(D10:D15)+SUM(F10:F15)+SUM(H10:H15)</f>
+        <v/>
+      </c>
+      <c r="C3" s="23" t="n"/>
+      <c r="D3" s="23" t="n"/>
+      <c r="E3" s="1" t="n"/>
+      <c r="F3" s="24">
+        <f>SUM(D16:D26)+SUM(F16:F26)+SUM(H16:H26)</f>
+        <v/>
+      </c>
+      <c r="G3" s="23" t="n"/>
+      <c r="H3" s="23" t="n"/>
+      <c r="I3" s="1" t="n"/>
+      <c r="J3" s="25">
+        <f>SUM(L10:L15)+SUM(N10:N15)+SUM(P10:P15)</f>
+        <v/>
+      </c>
+      <c r="K3" s="23" t="n"/>
+      <c r="L3" s="23" t="n"/>
+      <c r="M3" s="1" t="n"/>
+      <c r="N3" s="25">
+        <f>SUM(L16:L26)+SUM(N16:N26)+SUM(P16:P26)</f>
+        <v/>
+      </c>
+      <c r="O3" s="23" t="n"/>
+      <c r="P3" s="23" t="n"/>
+    </row>
+    <row r="4" ht="13" customHeight="1">
+      <c r="A4" s="1" t="n"/>
+      <c r="B4" s="26" t="inlineStr">
+        <is>
+          <t>40'RH stock</t>
+        </is>
+      </c>
+      <c r="C4" s="23" t="n"/>
+      <c r="D4" s="23" t="n"/>
+      <c r="E4" s="1" t="n"/>
+      <c r="F4" s="26" t="inlineStr">
+        <is>
+          <t>40'RH stock</t>
+        </is>
+      </c>
+      <c r="G4" s="23" t="n"/>
+      <c r="H4" s="23" t="n"/>
+      <c r="I4" s="1" t="n"/>
+      <c r="J4" s="26" t="inlineStr">
+        <is>
+          <t>40'RH stock</t>
+        </is>
+      </c>
+      <c r="K4" s="23" t="n"/>
+      <c r="L4" s="23" t="n"/>
+      <c r="M4" s="1" t="n"/>
+      <c r="N4" s="26" t="inlineStr">
+        <is>
+          <t>40'RH stock</t>
+        </is>
+      </c>
+      <c r="O4" s="23" t="n"/>
+      <c r="P4" s="23" t="n"/>
+    </row>
+    <row r="5" ht="13" customHeight="1">
+      <c r="A5" s="1" t="n"/>
+      <c r="B5" s="1" t="n"/>
+      <c r="C5" s="1" t="n"/>
+      <c r="D5" s="1" t="n"/>
+      <c r="E5" s="1" t="n"/>
+      <c r="F5" s="1" t="n"/>
+      <c r="G5" s="1" t="n"/>
+      <c r="H5" s="1" t="n"/>
+      <c r="I5" s="1" t="n"/>
+      <c r="J5" s="1" t="n"/>
+      <c r="K5" s="1" t="n"/>
+      <c r="L5" s="1" t="n"/>
+      <c r="M5" s="1" t="n"/>
+      <c r="N5" s="1" t="n"/>
+      <c r="O5" s="1" t="n"/>
+      <c r="P5" s="1" t="n"/>
+    </row>
+    <row r="6" ht="13" customHeight="1">
+      <c r="A6" s="1" t="n"/>
+      <c r="B6" s="1" t="n"/>
+      <c r="C6" s="1" t="n"/>
+      <c r="D6" s="1" t="n"/>
+      <c r="E6" s="1" t="n"/>
+      <c r="F6" s="1" t="n"/>
+      <c r="G6" s="1" t="n"/>
+      <c r="H6" s="1" t="n"/>
+      <c r="I6" s="1" t="n"/>
+      <c r="J6" s="1" t="n"/>
+      <c r="K6" s="1" t="n"/>
+      <c r="L6" s="1" t="n"/>
+      <c r="M6" s="1" t="n"/>
+      <c r="N6" s="1" t="n"/>
+      <c r="O6" s="1" t="n"/>
+      <c r="P6" s="1" t="n"/>
+    </row>
+    <row r="7" ht="13" customHeight="1">
+      <c r="A7" s="1" t="n"/>
+      <c r="B7" s="3" t="inlineStr">
+        <is>
+          <t>BKK27 / BC2  —  Stock by Built Year x Brand x Size</t>
+        </is>
+      </c>
+      <c r="C7" s="56" t="n"/>
+      <c r="D7" s="56" t="n"/>
+      <c r="E7" s="56" t="n"/>
+      <c r="F7" s="56" t="n"/>
+      <c r="G7" s="56" t="n"/>
+      <c r="H7" s="57" t="n"/>
+      <c r="I7" s="1" t="n"/>
+      <c r="J7" s="3" t="inlineStr">
+        <is>
+          <t>LCH27 / HAST  —  Stock by Built Year x Brand x Size</t>
+        </is>
+      </c>
+      <c r="K7" s="56" t="n"/>
+      <c r="L7" s="56" t="n"/>
+      <c r="M7" s="56" t="n"/>
+      <c r="N7" s="56" t="n"/>
+      <c r="O7" s="56" t="n"/>
+      <c r="P7" s="57" t="n"/>
+    </row>
+    <row r="8" ht="26" customHeight="1">
+      <c r="A8" s="1" t="n"/>
+      <c r="B8" s="18" t="inlineStr">
+        <is>
+          <t>YEAR
+BUILT</t>
+        </is>
+      </c>
+      <c r="C8" s="4" t="inlineStr">
+        <is>
+          <t>CARRIER</t>
+        </is>
+      </c>
+      <c r="D8" s="57" t="n"/>
+      <c r="E8" s="4" t="inlineStr">
+        <is>
+          <t>DAIKIN</t>
+        </is>
+      </c>
+      <c r="F8" s="57" t="n"/>
+      <c r="G8" s="4" t="inlineStr">
+        <is>
+          <t>THERMO KING</t>
+        </is>
+      </c>
+      <c r="H8" s="57" t="n"/>
+      <c r="I8" s="1" t="n"/>
+      <c r="J8" s="18" t="inlineStr">
+        <is>
+          <t>YEAR
+BUILT</t>
+        </is>
+      </c>
+      <c r="K8" s="4" t="inlineStr">
+        <is>
+          <t>CARRIER</t>
+        </is>
+      </c>
+      <c r="L8" s="57" t="n"/>
+      <c r="M8" s="4" t="inlineStr">
+        <is>
+          <t>DAIKIN</t>
+        </is>
+      </c>
+      <c r="N8" s="57" t="n"/>
+      <c r="O8" s="4" t="inlineStr">
+        <is>
+          <t>THERMO KING</t>
+        </is>
+      </c>
+      <c r="P8" s="57" t="n"/>
+    </row>
+    <row r="9" ht="13" customHeight="1">
+      <c r="A9" s="1" t="n"/>
+      <c r="B9" s="60" t="n"/>
+      <c r="C9" s="28" t="inlineStr">
+        <is>
+          <t>20'RE</t>
+        </is>
+      </c>
+      <c r="D9" s="28" t="inlineStr">
+        <is>
+          <t>40'RH</t>
+        </is>
+      </c>
+      <c r="E9" s="28" t="inlineStr">
+        <is>
+          <t>20'RE</t>
+        </is>
+      </c>
+      <c r="F9" s="28" t="inlineStr">
+        <is>
+          <t>40'RH</t>
+        </is>
+      </c>
+      <c r="G9" s="28" t="inlineStr">
+        <is>
+          <t>20'RE</t>
+        </is>
+      </c>
+      <c r="H9" s="28" t="inlineStr">
+        <is>
+          <t>40'RH</t>
+        </is>
+      </c>
+      <c r="I9" s="1" t="n"/>
+      <c r="J9" s="60" t="n"/>
+      <c r="K9" s="28" t="inlineStr">
+        <is>
+          <t>20'RE</t>
+        </is>
+      </c>
+      <c r="L9" s="28" t="inlineStr">
+        <is>
+          <t>40'RH</t>
+        </is>
+      </c>
+      <c r="M9" s="28" t="inlineStr">
+        <is>
+          <t>20'RE</t>
+        </is>
+      </c>
+      <c r="N9" s="28" t="inlineStr">
+        <is>
+          <t>40'RH</t>
+        </is>
+      </c>
+      <c r="O9" s="28" t="inlineStr">
+        <is>
+          <t>20'RE</t>
+        </is>
+      </c>
+      <c r="P9" s="28" t="inlineStr">
+        <is>
+          <t>40'RH</t>
+        </is>
+      </c>
+    </row>
+    <row r="10" ht="13" customHeight="1">
+      <c r="A10" s="1" t="n"/>
+      <c r="B10" s="29" t="n">
+        <v>2026</v>
+      </c>
+      <c r="C10" s="30" t="n"/>
+      <c r="D10" s="30" t="n"/>
+      <c r="E10" s="30" t="n"/>
+      <c r="F10" s="30" t="n"/>
+      <c r="G10" s="30" t="n"/>
+      <c r="H10" s="30" t="n"/>
+      <c r="I10" s="1" t="n"/>
+      <c r="J10" s="29" t="n">
+        <v>2026</v>
+      </c>
+      <c r="K10" s="30" t="n"/>
+      <c r="L10" s="30" t="n"/>
+      <c r="M10" s="30" t="n"/>
+      <c r="N10" s="30" t="n"/>
+      <c r="O10" s="30" t="n"/>
+      <c r="P10" s="30" t="n"/>
+    </row>
+    <row r="11" ht="13" customHeight="1">
+      <c r="A11" s="1" t="n"/>
+      <c r="B11" s="29" t="n">
+        <v>2025</v>
+      </c>
+      <c r="C11" s="30" t="n"/>
+      <c r="D11" s="30" t="n">
+        <v>3</v>
+      </c>
+      <c r="E11" s="30" t="n">
+        <v>2</v>
+      </c>
+      <c r="F11" s="30" t="n"/>
+      <c r="G11" s="30" t="n"/>
+      <c r="H11" s="30" t="n">
+        <v>1</v>
+      </c>
+      <c r="I11" s="1" t="n"/>
+      <c r="J11" s="29" t="n">
+        <v>2025</v>
+      </c>
+      <c r="K11" s="30" t="n"/>
+      <c r="L11" s="30" t="n">
+        <v>8</v>
+      </c>
+      <c r="M11" s="30" t="n"/>
+      <c r="N11" s="30" t="n"/>
+      <c r="O11" s="30" t="n"/>
+      <c r="P11" s="30" t="n"/>
+    </row>
+    <row r="12" ht="13" customHeight="1">
+      <c r="A12" s="1" t="n"/>
+      <c r="B12" s="29" t="n">
+        <v>2024</v>
+      </c>
+      <c r="C12" s="30" t="n"/>
+      <c r="D12" s="30" t="n"/>
+      <c r="E12" s="30" t="n"/>
+      <c r="F12" s="30" t="n"/>
+      <c r="G12" s="30" t="n"/>
+      <c r="H12" s="30" t="n"/>
+      <c r="I12" s="1" t="n"/>
+      <c r="J12" s="29" t="n">
+        <v>2024</v>
+      </c>
+      <c r="K12" s="30" t="n"/>
+      <c r="L12" s="30" t="n"/>
+      <c r="M12" s="30" t="n"/>
+      <c r="N12" s="30" t="n"/>
+      <c r="O12" s="30" t="n"/>
+      <c r="P12" s="30" t="n"/>
+    </row>
+    <row r="13" ht="13" customHeight="1">
+      <c r="A13" s="1" t="n"/>
+      <c r="B13" s="29" t="n">
+        <v>2023</v>
+      </c>
+      <c r="C13" s="30" t="n"/>
+      <c r="D13" s="30" t="n">
+        <v>1</v>
+      </c>
+      <c r="E13" s="30" t="n"/>
+      <c r="F13" s="30" t="n"/>
+      <c r="G13" s="30" t="n"/>
+      <c r="H13" s="30" t="n"/>
+      <c r="I13" s="1" t="n"/>
+      <c r="J13" s="29" t="n">
+        <v>2023</v>
+      </c>
+      <c r="K13" s="30" t="n"/>
+      <c r="L13" s="30" t="n">
+        <v>2</v>
+      </c>
+      <c r="M13" s="30" t="n"/>
+      <c r="N13" s="30" t="n"/>
+      <c r="O13" s="30" t="n"/>
+      <c r="P13" s="30" t="n"/>
+    </row>
+    <row r="14" ht="13" customHeight="1">
+      <c r="A14" s="1" t="n"/>
+      <c r="B14" s="29" t="n">
+        <v>2022</v>
+      </c>
+      <c r="C14" s="30" t="n"/>
+      <c r="D14" s="30" t="n"/>
+      <c r="E14" s="30" t="n"/>
+      <c r="F14" s="30" t="n"/>
+      <c r="G14" s="30" t="n"/>
+      <c r="H14" s="30" t="n"/>
+      <c r="I14" s="1" t="n"/>
+      <c r="J14" s="29" t="n">
+        <v>2022</v>
+      </c>
+      <c r="K14" s="30" t="n"/>
+      <c r="L14" s="30" t="n"/>
+      <c r="M14" s="30" t="n"/>
+      <c r="N14" s="30" t="n"/>
+      <c r="O14" s="30" t="n"/>
+      <c r="P14" s="30" t="n"/>
+    </row>
+    <row r="15" ht="13" customHeight="1">
+      <c r="A15" s="1" t="n"/>
+      <c r="B15" s="29" t="n">
+        <v>2021</v>
+      </c>
+      <c r="C15" s="30" t="n">
+        <v>8</v>
+      </c>
+      <c r="D15" s="30" t="n">
+        <v>6</v>
+      </c>
+      <c r="E15" s="30" t="n"/>
+      <c r="F15" s="30" t="n"/>
+      <c r="G15" s="30" t="n"/>
+      <c r="H15" s="30" t="n"/>
+      <c r="I15" s="1" t="n"/>
+      <c r="J15" s="29" t="n">
+        <v>2021</v>
+      </c>
+      <c r="K15" s="30" t="n">
+        <v>2</v>
+      </c>
+      <c r="L15" s="30" t="n">
+        <v>3</v>
+      </c>
+      <c r="M15" s="30" t="n"/>
+      <c r="N15" s="30" t="n"/>
+      <c r="O15" s="30" t="n"/>
+      <c r="P15" s="30" t="n"/>
+    </row>
+    <row r="16" ht="13" customHeight="1">
+      <c r="A16" s="1" t="n"/>
+      <c r="B16" s="31" t="n">
+        <v>2020</v>
+      </c>
+      <c r="C16" s="32" t="n">
+        <v>1</v>
+      </c>
+      <c r="D16" s="32" t="n">
+        <v>5</v>
+      </c>
+      <c r="E16" s="32" t="n"/>
+      <c r="F16" s="32" t="n"/>
+      <c r="G16" s="32" t="n"/>
+      <c r="H16" s="32" t="n"/>
+      <c r="I16" s="1" t="n"/>
+      <c r="J16" s="31" t="n">
+        <v>2020</v>
+      </c>
+      <c r="K16" s="32" t="n"/>
+      <c r="L16" s="32" t="n">
+        <v>11</v>
+      </c>
+      <c r="M16" s="32" t="n"/>
+      <c r="N16" s="32" t="n"/>
+      <c r="O16" s="32" t="n"/>
+      <c r="P16" s="32" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="17" ht="13" customHeight="1">
+      <c r="A17" s="1" t="n"/>
+      <c r="B17" s="31" t="n">
+        <v>2019</v>
+      </c>
+      <c r="C17" s="32" t="n">
+        <v>3</v>
+      </c>
+      <c r="D17" s="32" t="n">
+        <v>5</v>
+      </c>
+      <c r="E17" s="32" t="n"/>
+      <c r="F17" s="32" t="n"/>
+      <c r="G17" s="32" t="n"/>
+      <c r="H17" s="32" t="n"/>
+      <c r="I17" s="1" t="n"/>
+      <c r="J17" s="31" t="n">
+        <v>2019</v>
+      </c>
+      <c r="K17" s="32" t="n"/>
+      <c r="L17" s="32" t="n">
+        <v>8</v>
+      </c>
+      <c r="M17" s="32" t="n"/>
+      <c r="N17" s="32" t="n"/>
+      <c r="O17" s="32" t="n"/>
+      <c r="P17" s="32" t="n"/>
+    </row>
+    <row r="18" ht="13" customHeight="1">
+      <c r="A18" s="1" t="n"/>
+      <c r="B18" s="31" t="n">
+        <v>2018</v>
+      </c>
+      <c r="C18" s="32" t="n">
+        <v>1</v>
+      </c>
+      <c r="D18" s="32" t="n"/>
+      <c r="E18" s="32" t="n"/>
+      <c r="F18" s="32" t="n"/>
+      <c r="G18" s="32" t="n"/>
+      <c r="H18" s="32" t="n"/>
+      <c r="I18" s="1" t="n"/>
+      <c r="J18" s="31" t="n">
+        <v>2018</v>
+      </c>
+      <c r="K18" s="32" t="n"/>
+      <c r="L18" s="32" t="n"/>
+      <c r="M18" s="32" t="n"/>
+      <c r="N18" s="32" t="n"/>
+      <c r="O18" s="32" t="n"/>
+      <c r="P18" s="32" t="n"/>
+    </row>
+    <row r="19" ht="13" customHeight="1">
+      <c r="A19" s="1" t="n"/>
+      <c r="B19" s="31" t="n">
+        <v>2017</v>
+      </c>
+      <c r="C19" s="32" t="n">
+        <v>2</v>
+      </c>
+      <c r="D19" s="32" t="n">
+        <v>1</v>
+      </c>
+      <c r="E19" s="32" t="n"/>
+      <c r="F19" s="32" t="n"/>
+      <c r="G19" s="32" t="n"/>
+      <c r="H19" s="32" t="n"/>
+      <c r="I19" s="1" t="n"/>
+      <c r="J19" s="31" t="n">
+        <v>2017</v>
+      </c>
+      <c r="K19" s="32" t="n">
+        <v>2</v>
+      </c>
+      <c r="L19" s="32" t="n">
+        <v>2</v>
+      </c>
+      <c r="M19" s="32" t="n"/>
+      <c r="N19" s="32" t="n"/>
+      <c r="O19" s="32" t="n"/>
+      <c r="P19" s="32" t="n"/>
+    </row>
+    <row r="20" ht="13" customHeight="1">
+      <c r="A20" s="1" t="n"/>
+      <c r="B20" s="31" t="n">
+        <v>2016</v>
+      </c>
+      <c r="C20" s="32" t="n">
+        <v>2</v>
+      </c>
+      <c r="D20" s="32" t="n">
+        <v>3</v>
+      </c>
+      <c r="E20" s="32" t="n">
+        <v>2</v>
+      </c>
+      <c r="F20" s="32" t="n"/>
+      <c r="G20" s="32" t="n"/>
+      <c r="H20" s="32" t="n"/>
+      <c r="I20" s="1" t="n"/>
+      <c r="J20" s="31" t="n">
+        <v>2016</v>
+      </c>
+      <c r="K20" s="32" t="n"/>
+      <c r="L20" s="32" t="n"/>
+      <c r="M20" s="32" t="n"/>
+      <c r="N20" s="32" t="n"/>
+      <c r="O20" s="32" t="n"/>
+      <c r="P20" s="32" t="n"/>
+    </row>
+    <row r="21" ht="13" customHeight="1">
+      <c r="A21" s="1" t="n"/>
+      <c r="B21" s="33" t="n">
+        <v>2015</v>
+      </c>
+      <c r="C21" s="34" t="n"/>
+      <c r="D21" s="34" t="n">
+        <v>3</v>
+      </c>
+      <c r="E21" s="34" t="n">
+        <v>2</v>
+      </c>
+      <c r="F21" s="34" t="n"/>
+      <c r="G21" s="34" t="n"/>
+      <c r="H21" s="34" t="n"/>
+      <c r="I21" s="1" t="n"/>
+      <c r="J21" s="33" t="n">
+        <v>2015</v>
+      </c>
+      <c r="K21" s="34" t="n"/>
+      <c r="L21" s="34" t="n">
+        <v>2</v>
+      </c>
+      <c r="M21" s="34" t="n"/>
+      <c r="N21" s="34" t="n"/>
+      <c r="O21" s="34" t="n"/>
+      <c r="P21" s="34" t="n"/>
+    </row>
+    <row r="22" ht="13" customHeight="1">
+      <c r="A22" s="1" t="n"/>
+      <c r="B22" s="33" t="n">
+        <v>2014</v>
+      </c>
+      <c r="C22" s="34" t="n">
+        <v>2</v>
+      </c>
+      <c r="D22" s="34" t="n"/>
+      <c r="E22" s="34" t="n"/>
+      <c r="F22" s="34" t="n"/>
+      <c r="G22" s="34" t="n"/>
+      <c r="H22" s="34" t="n"/>
+      <c r="I22" s="1" t="n"/>
+      <c r="J22" s="33" t="n">
+        <v>2014</v>
+      </c>
+      <c r="K22" s="34" t="n"/>
+      <c r="L22" s="34" t="n">
+        <v>5</v>
+      </c>
+      <c r="M22" s="34" t="n"/>
+      <c r="N22" s="34" t="n"/>
+      <c r="O22" s="34" t="n"/>
+      <c r="P22" s="34" t="n"/>
+    </row>
+    <row r="23" ht="13" customHeight="1">
+      <c r="A23" s="1" t="n"/>
+      <c r="B23" s="33" t="n">
+        <v>2013</v>
+      </c>
+      <c r="C23" s="34" t="n">
+        <v>1</v>
+      </c>
+      <c r="D23" s="34" t="n"/>
+      <c r="E23" s="34" t="n">
+        <v>4</v>
+      </c>
+      <c r="F23" s="34" t="n">
+        <v>3</v>
+      </c>
+      <c r="G23" s="34" t="n">
+        <v>2</v>
+      </c>
+      <c r="H23" s="34" t="n">
+        <v>1</v>
+      </c>
+      <c r="I23" s="1" t="n"/>
+      <c r="J23" s="33" t="n">
+        <v>2013</v>
+      </c>
+      <c r="K23" s="34" t="n"/>
+      <c r="L23" s="34" t="n"/>
+      <c r="M23" s="34" t="n">
+        <v>2</v>
+      </c>
+      <c r="N23" s="34" t="n">
+        <v>2</v>
+      </c>
+      <c r="O23" s="34" t="n"/>
+      <c r="P23" s="34" t="n"/>
+    </row>
+    <row r="24" ht="13" customHeight="1">
+      <c r="A24" s="1" t="n"/>
+      <c r="B24" s="33" t="n">
+        <v>2012</v>
+      </c>
+      <c r="C24" s="34" t="n">
+        <v>1</v>
+      </c>
+      <c r="D24" s="34" t="n">
+        <v>2</v>
+      </c>
+      <c r="E24" s="34" t="n"/>
+      <c r="F24" s="34" t="n"/>
+      <c r="G24" s="34" t="n"/>
+      <c r="H24" s="34" t="n"/>
+      <c r="I24" s="1" t="n"/>
+      <c r="J24" s="33" t="n">
+        <v>2012</v>
+      </c>
+      <c r="K24" s="34" t="n"/>
+      <c r="L24" s="34" t="n">
+        <v>3</v>
+      </c>
+      <c r="M24" s="34" t="n">
+        <v>1</v>
+      </c>
+      <c r="N24" s="34" t="n"/>
+      <c r="O24" s="34" t="n"/>
+      <c r="P24" s="34" t="n"/>
+    </row>
+    <row r="25" ht="13" customHeight="1">
+      <c r="A25" s="1" t="n"/>
+      <c r="B25" s="33" t="n">
+        <v>2011</v>
+      </c>
+      <c r="C25" s="34" t="n"/>
+      <c r="D25" s="34" t="n"/>
+      <c r="E25" s="34" t="n"/>
+      <c r="F25" s="34" t="n">
+        <v>3</v>
+      </c>
+      <c r="G25" s="34" t="n"/>
+      <c r="H25" s="34" t="n"/>
+      <c r="I25" s="1" t="n"/>
+      <c r="J25" s="33" t="n">
+        <v>2011</v>
+      </c>
+      <c r="K25" s="34" t="n"/>
+      <c r="L25" s="34" t="n"/>
+      <c r="M25" s="34" t="n"/>
+      <c r="N25" s="34" t="n">
+        <v>5</v>
+      </c>
+      <c r="O25" s="34" t="n"/>
+      <c r="P25" s="34" t="n"/>
+    </row>
+    <row r="26" ht="13" customHeight="1">
+      <c r="A26" s="1" t="n"/>
+      <c r="B26" s="35" t="n">
+        <v>2010</v>
+      </c>
+      <c r="C26" s="36" t="n"/>
+      <c r="D26" s="36" t="n">
+        <v>1</v>
+      </c>
+      <c r="E26" s="36" t="n"/>
+      <c r="F26" s="36" t="n"/>
+      <c r="G26" s="36" t="n"/>
+      <c r="H26" s="36" t="n"/>
+      <c r="I26" s="1" t="n"/>
+      <c r="J26" s="35" t="n">
+        <v>2010</v>
+      </c>
+      <c r="K26" s="36" t="n"/>
+      <c r="L26" s="36" t="n">
+        <v>1</v>
+      </c>
+      <c r="M26" s="36" t="n"/>
+      <c r="N26" s="36" t="n"/>
+      <c r="O26" s="36" t="n"/>
+      <c r="P26" s="36" t="n"/>
+    </row>
+    <row r="27" ht="13" customHeight="1">
+      <c r="A27" s="1" t="n"/>
+      <c r="B27" s="13" t="inlineStr">
+        <is>
+          <t>GTTL</t>
+        </is>
+      </c>
+      <c r="C27" s="13" t="n">
+        <v>21</v>
+      </c>
+      <c r="D27" s="13" t="n">
+        <v>30</v>
+      </c>
+      <c r="E27" s="13" t="n">
+        <v>10</v>
+      </c>
+      <c r="F27" s="13" t="n">
+        <v>6</v>
+      </c>
+      <c r="G27" s="13" t="n">
+        <v>2</v>
+      </c>
+      <c r="H27" s="13" t="n">
+        <v>2</v>
+      </c>
+      <c r="I27" s="1" t="n"/>
+      <c r="J27" s="13" t="inlineStr">
+        <is>
+          <t>GTTL</t>
+        </is>
+      </c>
+      <c r="K27" s="13" t="n">
+        <v>4</v>
+      </c>
+      <c r="L27" s="13" t="n">
+        <v>45</v>
+      </c>
+      <c r="M27" s="13" t="n">
+        <v>3</v>
+      </c>
+      <c r="N27" s="13" t="n">
+        <v>7</v>
+      </c>
+      <c r="O27" s="13" t="n"/>
+      <c r="P27" s="13" t="n">
+        <v>1</v>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="10">
+    <mergeCell ref="K8:L8"/>
+    <mergeCell ref="J8:J9"/>
+    <mergeCell ref="E8:F8"/>
+    <mergeCell ref="B8:B9"/>
+    <mergeCell ref="B7:H7"/>
+    <mergeCell ref="J7:P7"/>
+    <mergeCell ref="G8:H8"/>
+    <mergeCell ref="M8:N8"/>
+    <mergeCell ref="C8:D8"/>
+    <mergeCell ref="O8:P8"/>
+  </mergeCells>
+  <printOptions horizontalCentered="1"/>
+  <pageMargins left="0.4" right="0.4" top="0.5" bottom="0.5" header="0.5" footer="0.5"/>
+  <pageSetup orientation="landscape" paperSize="9" fitToHeight="1" fitToWidth="1"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -8158,14 +8128,14 @@
     <row r="33" ht="13" customHeight="1">
       <c r="A33" s="1" t="n"/>
       <c r="B33" s="53">
-        <f>SUM('TOTAL RH'!D42:D48)+SUM('TOTAL RH'!F42:F48)+SUM('TOTAL RH'!H42:H48)</f>
+        <f>SUM('YEAR BUILT'!D10:D16)+SUM('YEAR BUILT'!F10:F16)+SUM('YEAR BUILT'!H10:H16)</f>
         <v/>
       </c>
       <c r="C33" s="23" t="n"/>
       <c r="D33" s="23" t="n"/>
       <c r="E33" s="1" t="n"/>
       <c r="F33" s="54">
-        <f>SUM('TOTAL RH'!L42:L48)+SUM('TOTAL RH'!N42:N48)+SUM('TOTAL RH'!P42:P48)</f>
+        <f>SUM('YEAR BUILT'!L10:L16)+SUM('YEAR BUILT'!N10:N16)+SUM('YEAR BUILT'!P10:P16)</f>
         <v/>
       </c>
       <c r="G33" s="23" t="n"/>
@@ -8267,28 +8237,28 @@
     <row r="37" ht="13" customHeight="1">
       <c r="A37" s="1" t="n"/>
       <c r="B37" s="53">
-        <f>'TOTAL RH'!B35</f>
+        <f>'YEAR BUILT'!B3</f>
         <v/>
       </c>
       <c r="C37" s="23" t="n"/>
       <c r="D37" s="23" t="n"/>
       <c r="E37" s="1" t="n"/>
       <c r="F37" s="53">
-        <f>'TOTAL RH'!F35</f>
+        <f>'YEAR BUILT'!F3</f>
         <v/>
       </c>
       <c r="G37" s="23" t="n"/>
       <c r="H37" s="23" t="n"/>
       <c r="I37" s="1" t="n"/>
       <c r="J37" s="54">
-        <f>'TOTAL RH'!J35</f>
+        <f>'YEAR BUILT'!J3</f>
         <v/>
       </c>
       <c r="K37" s="23" t="n"/>
       <c r="L37" s="23" t="n"/>
       <c r="M37" s="1" t="n"/>
       <c r="N37" s="54">
-        <f>'TOTAL RH'!N35</f>
+        <f>'YEAR BUILT'!N3</f>
         <v/>
       </c>
       <c r="O37" s="23" t="n"/>
@@ -8414,11 +8384,11 @@
         </is>
       </c>
       <c r="C42" s="50">
-        <f>'TOTAL RH'!C59</f>
+        <f>'YEAR BUILT'!C27</f>
         <v/>
       </c>
       <c r="D42" s="50">
-        <f>'TOTAL RH'!D59</f>
+        <f>'YEAR BUILT'!D27</f>
         <v/>
       </c>
       <c r="E42" s="1" t="n"/>
@@ -8430,11 +8400,11 @@
         </is>
       </c>
       <c r="I42" s="50">
-        <f>'TOTAL RH'!K59</f>
+        <f>'YEAR BUILT'!K27</f>
         <v/>
       </c>
       <c r="J42" s="50">
-        <f>'TOTAL RH'!L59</f>
+        <f>'YEAR BUILT'!L27</f>
         <v/>
       </c>
       <c r="K42" s="1" t="n"/>
@@ -8452,11 +8422,11 @@
         </is>
       </c>
       <c r="C43" s="50">
-        <f>'TOTAL RH'!E59</f>
+        <f>'YEAR BUILT'!E27</f>
         <v/>
       </c>
       <c r="D43" s="50">
-        <f>'TOTAL RH'!F59</f>
+        <f>'YEAR BUILT'!F27</f>
         <v/>
       </c>
       <c r="E43" s="1" t="n"/>
@@ -8468,11 +8438,11 @@
         </is>
       </c>
       <c r="I43" s="50">
-        <f>'TOTAL RH'!M59</f>
+        <f>'YEAR BUILT'!M27</f>
         <v/>
       </c>
       <c r="J43" s="50">
-        <f>'TOTAL RH'!N59</f>
+        <f>'YEAR BUILT'!N27</f>
         <v/>
       </c>
       <c r="K43" s="1" t="n"/>
@@ -8490,11 +8460,11 @@
         </is>
       </c>
       <c r="C44" s="50">
-        <f>'TOTAL RH'!G59</f>
+        <f>'YEAR BUILT'!G27</f>
         <v/>
       </c>
       <c r="D44" s="50">
-        <f>'TOTAL RH'!H59</f>
+        <f>'YEAR BUILT'!H27</f>
         <v/>
       </c>
       <c r="E44" s="1" t="n"/>
@@ -8506,11 +8476,11 @@
         </is>
       </c>
       <c r="I44" s="50">
-        <f>'TOTAL RH'!O59</f>
+        <f>'YEAR BUILT'!O27</f>
         <v/>
       </c>
       <c r="J44" s="50">
-        <f>'TOTAL RH'!P59</f>
+        <f>'YEAR BUILT'!P27</f>
         <v/>
       </c>
       <c r="K44" s="1" t="n"/>
@@ -8542,7 +8512,7 @@
       <c r="A46" s="1" t="n"/>
       <c r="B46" s="55" t="inlineStr">
         <is>
-          <t>Full 2010-2026 Year x Brand x Size breakdown is on the TOTAL RH sheet.</t>
+          <t>Full 2010-2026 Year x Brand x Size breakdown is on the YEAR BUILT sheet.</t>
         </is>
       </c>
       <c r="C46" s="1" t="n"/>

</xml_diff>

<commit_message>
TOTAL RH: columns B and H = 165 px; fix pixel-width conversion
User spec: label columns B and H on TOTAL RH are 165 px wide.
Also fixes an earlier mistake: the stored column width attribute is
pixels/7 for Calibri 11 (Excel's UI width is that minus 5/7), so the
B-Q "61 px" from 2026-10-05 had been stored as 8.0 = 56 px. Now
stored as 61/7 so columns really are 61 px; verified by converting the
saved widths back to pixels.

Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Stock_Daily_Reefer_10-8.xlsx
+++ b/Stock_Daily_Reefer_10-8.xlsx
@@ -5231,22 +5231,22 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="4" customWidth="1" min="1" max="1"/>
-    <col width="8" customWidth="1" min="2" max="2"/>
-    <col width="8" customWidth="1" min="3" max="3"/>
-    <col width="8" customWidth="1" min="4" max="4"/>
-    <col width="8" customWidth="1" min="5" max="5"/>
-    <col width="8" customWidth="1" min="6" max="6"/>
-    <col width="8" customWidth="1" min="7" max="7"/>
-    <col width="8" customWidth="1" min="8" max="8"/>
-    <col width="8" customWidth="1" min="9" max="9"/>
-    <col width="8" customWidth="1" min="10" max="10"/>
-    <col width="8" customWidth="1" min="11" max="11"/>
-    <col width="8" customWidth="1" min="12" max="12"/>
-    <col width="8" customWidth="1" min="13" max="13"/>
-    <col width="8" customWidth="1" min="14" max="14"/>
-    <col width="8" customWidth="1" min="15" max="15"/>
-    <col width="8" customWidth="1" min="16" max="16"/>
-    <col width="8" customWidth="1" min="17" max="17"/>
+    <col width="23.57142857142857" customWidth="1" min="2" max="2"/>
+    <col width="8.714285714285714" customWidth="1" min="3" max="3"/>
+    <col width="8.714285714285714" customWidth="1" min="4" max="4"/>
+    <col width="8.714285714285714" customWidth="1" min="5" max="5"/>
+    <col width="8.714285714285714" customWidth="1" min="6" max="6"/>
+    <col width="8.714285714285714" customWidth="1" min="7" max="7"/>
+    <col width="23.57142857142857" customWidth="1" min="8" max="8"/>
+    <col width="8.714285714285714" customWidth="1" min="9" max="9"/>
+    <col width="8.714285714285714" customWidth="1" min="10" max="10"/>
+    <col width="8.714285714285714" customWidth="1" min="11" max="11"/>
+    <col width="8.714285714285714" customWidth="1" min="12" max="12"/>
+    <col width="8.714285714285714" customWidth="1" min="13" max="13"/>
+    <col width="8.714285714285714" customWidth="1" min="14" max="14"/>
+    <col width="8.714285714285714" customWidth="1" min="15" max="15"/>
+    <col width="8.714285714285714" customWidth="1" min="16" max="16"/>
+    <col width="8.714285714285714" customWidth="1" min="17" max="17"/>
   </cols>
   <sheetData>
     <row r="1" ht="13" customHeight="1">
@@ -6396,22 +6396,22 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="4" customWidth="1" min="1" max="1"/>
-    <col width="8" customWidth="1" min="2" max="2"/>
-    <col width="8" customWidth="1" min="3" max="3"/>
-    <col width="8" customWidth="1" min="4" max="4"/>
-    <col width="8" customWidth="1" min="5" max="5"/>
-    <col width="8" customWidth="1" min="6" max="6"/>
-    <col width="8" customWidth="1" min="7" max="7"/>
-    <col width="8" customWidth="1" min="8" max="8"/>
-    <col width="8" customWidth="1" min="9" max="9"/>
-    <col width="8" customWidth="1" min="10" max="10"/>
-    <col width="8" customWidth="1" min="11" max="11"/>
-    <col width="8" customWidth="1" min="12" max="12"/>
-    <col width="8" customWidth="1" min="13" max="13"/>
-    <col width="8" customWidth="1" min="14" max="14"/>
-    <col width="8" customWidth="1" min="15" max="15"/>
-    <col width="8" customWidth="1" min="16" max="16"/>
-    <col width="8" customWidth="1" min="17" max="17"/>
+    <col width="8.714285714285714" customWidth="1" min="2" max="2"/>
+    <col width="8.714285714285714" customWidth="1" min="3" max="3"/>
+    <col width="8.714285714285714" customWidth="1" min="4" max="4"/>
+    <col width="8.714285714285714" customWidth="1" min="5" max="5"/>
+    <col width="8.714285714285714" customWidth="1" min="6" max="6"/>
+    <col width="8.714285714285714" customWidth="1" min="7" max="7"/>
+    <col width="8.714285714285714" customWidth="1" min="8" max="8"/>
+    <col width="8.714285714285714" customWidth="1" min="9" max="9"/>
+    <col width="8.714285714285714" customWidth="1" min="10" max="10"/>
+    <col width="8.714285714285714" customWidth="1" min="11" max="11"/>
+    <col width="8.714285714285714" customWidth="1" min="12" max="12"/>
+    <col width="8.714285714285714" customWidth="1" min="13" max="13"/>
+    <col width="8.714285714285714" customWidth="1" min="14" max="14"/>
+    <col width="8.714285714285714" customWidth="1" min="15" max="15"/>
+    <col width="8.714285714285714" customWidth="1" min="16" max="16"/>
+    <col width="8.714285714285714" customWidth="1" min="17" max="17"/>
   </cols>
   <sheetData>
     <row r="1" ht="13" customHeight="1">

</xml_diff>